<commit_message>
Corrected 15rs Jar + Imli
</commit_message>
<xml_diff>
--- a/assets/Sweet_Crush_Gold_Rate_List.xlsx
+++ b/assets/Sweet_Crush_Gold_Rate_List.xlsx
@@ -8,32 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Documents\SweetCrushGoldSite\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92336F49-A1D9-4045-A4C1-CC1438F7CE75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{403BFDF3-7E04-486A-923F-DE7FFC8DF49A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Rate List" sheetId="2" r:id="rId1"/>
+    <sheet name="Rate List" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="67">
   <si>
     <t>Dear All Distributers, Update the Trader Price List</t>
   </si>
@@ -56,178 +43,184 @@
     <t>Trade Price</t>
   </si>
   <si>
+    <t>Sawad Candy Box</t>
+  </si>
+  <si>
+    <t>36x50</t>
+  </si>
+  <si>
     <t>Mix Fruit Toffee Jar</t>
   </si>
   <si>
+    <t>30x150</t>
+  </si>
+  <si>
     <t>Khoya Toffee</t>
   </si>
   <si>
+    <t>48x30</t>
+  </si>
+  <si>
     <t>Khoya Badam</t>
   </si>
   <si>
+    <t>48x15</t>
+  </si>
+  <si>
     <t>Cone Jelly Jar</t>
   </si>
   <si>
+    <t>12x80</t>
+  </si>
+  <si>
+    <t>Cornoto Cone Chocolate</t>
+  </si>
+  <si>
+    <t>24x30</t>
+  </si>
+  <si>
     <t>Egg Tweet</t>
   </si>
   <si>
     <t>Won Chocolate Paste Jar</t>
   </si>
   <si>
+    <t>27x80</t>
+  </si>
+  <si>
     <t>Shami Meva</t>
   </si>
   <si>
     <t>Desi Anda</t>
   </si>
   <si>
+    <t>24x60</t>
+  </si>
+  <si>
+    <t>Yumz</t>
+  </si>
+  <si>
+    <t>24x24</t>
+  </si>
+  <si>
     <t>Fudge Toffee Jar</t>
   </si>
   <si>
+    <t>2 Ever Bunty Sheet</t>
+  </si>
+  <si>
+    <t>60x30</t>
+  </si>
+  <si>
     <t>Silk + Bubly Chocolate</t>
   </si>
   <si>
+    <t>30x30</t>
+  </si>
+  <si>
     <t>Daily Milk Chocolate</t>
   </si>
   <si>
     <t>Spoon Chocolate</t>
   </si>
   <si>
+    <t>36x30</t>
+  </si>
+  <si>
+    <t>4 Ever Sheet Bunty</t>
+  </si>
+  <si>
     <t>Badam Candy</t>
   </si>
   <si>
     <t>Sorbon Mini Cone Chocolate</t>
   </si>
   <si>
+    <t>Choco-Crunch</t>
+  </si>
+  <si>
+    <t>24x18</t>
+  </si>
+  <si>
+    <t>Tim Tim Imli Box</t>
+  </si>
+  <si>
+    <t>Usailah Cup Imli</t>
+  </si>
+  <si>
+    <t>30x12</t>
+  </si>
+  <si>
     <t>Lolipop Pop On</t>
   </si>
   <si>
+    <t>18x50</t>
+  </si>
+  <si>
+    <t>Liquid Chocolate Silk</t>
+  </si>
+  <si>
+    <t>Umberala Chocolate</t>
+  </si>
+  <si>
+    <t>Sweeto Chocolate Balls</t>
+  </si>
+  <si>
+    <t>36x60</t>
+  </si>
+  <si>
+    <t>Nimko Halla Gula</t>
+  </si>
+  <si>
+    <t>12x6</t>
+  </si>
+  <si>
+    <t>Usailah AnarDana Imli</t>
+  </si>
+  <si>
+    <t>Sweeto Chocolate Balls Jar</t>
+  </si>
+  <si>
+    <t>18x80</t>
+  </si>
+  <si>
+    <t>Bano Nimko</t>
+  </si>
+  <si>
+    <t>Feeder</t>
+  </si>
+  <si>
+    <t>Bottle Candy (Magic Can)</t>
+  </si>
+  <si>
+    <t>Sting + Zombiez Bubble</t>
+  </si>
+  <si>
+    <t>12x120</t>
+  </si>
+  <si>
+    <t>Love Candy 100 pc</t>
+  </si>
+  <si>
+    <t>16x100</t>
+  </si>
+  <si>
+    <t>Love Candy 60 pc</t>
+  </si>
+  <si>
+    <t>30x60</t>
+  </si>
+  <si>
     <t>Regards:-       A.R Enterprises, Lahore</t>
   </si>
   <si>
-    <t>36x50</t>
-  </si>
-  <si>
-    <t>Cornoto Cone Chocolate</t>
-  </si>
-  <si>
-    <t>24x24</t>
-  </si>
-  <si>
-    <t>30x30</t>
-  </si>
-  <si>
-    <t>4 Ever Sheet Bunty</t>
-  </si>
-  <si>
-    <t>Tim Tim Imli Box</t>
-  </si>
-  <si>
-    <t>24x18</t>
-  </si>
-  <si>
-    <t>Liquid Chocolate Silk</t>
-  </si>
-  <si>
-    <t>24x30</t>
-  </si>
-  <si>
-    <t>Sawad Candy Box</t>
-  </si>
-  <si>
-    <t>2 Ever Bunty Sheet</t>
-  </si>
-  <si>
-    <t>Umberala Chocolate</t>
-  </si>
-  <si>
-    <t>30x150</t>
-  </si>
-  <si>
-    <t>48x30</t>
-  </si>
-  <si>
-    <t>Sweeto Chocolate Balls</t>
-  </si>
-  <si>
-    <t>18x50</t>
-  </si>
-  <si>
-    <t>30x12</t>
-  </si>
-  <si>
-    <t>36x30</t>
-  </si>
-  <si>
-    <t>24x60</t>
-  </si>
-  <si>
-    <t>27x80</t>
-  </si>
-  <si>
-    <t>48x15</t>
-  </si>
-  <si>
-    <t>Nimko Halla Gula</t>
-  </si>
-  <si>
-    <t>12x6</t>
-  </si>
-  <si>
-    <t>Bano Nimko</t>
-  </si>
-  <si>
-    <t>60x30</t>
-  </si>
-  <si>
-    <t>Usailah Cup Imli</t>
-  </si>
-  <si>
-    <t>Usailah AnarDana Imli</t>
-  </si>
-  <si>
-    <t>Sweeto Chocolate Balls Jar</t>
-  </si>
-  <si>
-    <t>18x80</t>
-  </si>
-  <si>
     <t>Note:-  (ONLY CASH No Credit Policy)</t>
   </si>
   <si>
-    <t>12x80</t>
-  </si>
-  <si>
-    <t>Yumz</t>
-  </si>
-  <si>
-    <t>Choco-Crunch</t>
-  </si>
-  <si>
-    <t>36x60</t>
-  </si>
-  <si>
-    <t>Feeder</t>
-  </si>
-  <si>
-    <t>Bottle Candy (Magic Can)</t>
-  </si>
-  <si>
-    <t>Sting + Zombiez Bubble</t>
-  </si>
-  <si>
-    <t>12x120</t>
-  </si>
-  <si>
-    <t>Love Candy 100 pc</t>
-  </si>
-  <si>
-    <t>16x100</t>
-  </si>
-  <si>
-    <t>Love Candy 60 pc</t>
-  </si>
-  <si>
-    <t>30x60</t>
+    <t>Mix Fruit Jelly Jar</t>
+  </si>
+  <si>
+    <t>9x50</t>
   </si>
 </sst>
 </file>
@@ -309,7 +302,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -341,11 +334,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -362,13 +392,22 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -585,8 +624,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AC6F22B-71DD-4ECC-A01A-5BEA50CE676C}">
-  <dimension ref="A1:F39"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F40"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24.36328125" bestFit="1" customWidth="1"/>
@@ -596,17 +635,17 @@
     <col min="6" max="6" width="10.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-    </row>
-    <row r="2" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+    </row>
+    <row r="2" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -626,15 +665,15 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="D3" s="1">
         <v>2</v>
@@ -646,15 +685,15 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="D4" s="1">
         <v>2</v>
@@ -666,15 +705,15 @@
         <v>260</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="D5" s="1">
         <v>5</v>
@@ -686,15 +725,15 @@
         <v>130</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="D6" s="1">
         <v>10</v>
@@ -706,15 +745,15 @@
         <v>130</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>53</v>
+        <v>16</v>
       </c>
       <c r="D7" s="1">
         <v>5</v>
@@ -726,15 +765,15 @@
         <v>350</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="D8" s="1">
         <v>5</v>
@@ -746,15 +785,15 @@
         <v>130</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="D9" s="1">
         <v>10</v>
@@ -766,15 +805,15 @@
         <v>260</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="D10" s="1">
         <v>5</v>
@@ -786,15 +825,15 @@
         <v>350</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="D11" s="1">
         <v>5</v>
@@ -806,15 +845,15 @@
         <v>130</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>10</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="D12" s="1">
         <v>5</v>
@@ -826,15 +865,15 @@
         <v>250</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D13" s="1">
         <v>10</v>
@@ -846,15 +885,15 @@
         <v>200</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="D14" s="1">
         <v>5</v>
@@ -866,15 +905,15 @@
         <v>260</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="D15" s="1">
         <v>5</v>
@@ -886,15 +925,15 @@
         <v>130</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D16" s="1">
         <v>10</v>
@@ -906,15 +945,15 @@
         <v>260</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D17" s="1">
         <v>10</v>
@@ -926,15 +965,15 @@
         <v>260</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>16</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D18" s="1">
         <v>10</v>
@@ -946,15 +985,15 @@
         <v>260</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>17</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="D19" s="1">
         <v>10</v>
@@ -966,15 +1005,15 @@
         <v>260</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>18</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D20" s="2">
         <v>5</v>
@@ -986,15 +1025,15 @@
         <v>130</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>19</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="D21" s="2">
         <v>10</v>
@@ -1006,15 +1045,15 @@
         <v>260</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
         <v>20</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="D22" s="2">
         <v>20</v>
@@ -1026,15 +1065,15 @@
         <v>300</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
         <v>21</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="D23" s="2">
         <v>20</v>
@@ -1046,15 +1085,15 @@
         <v>320</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3">
         <v>22</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D24" s="2">
         <v>60</v>
@@ -1066,15 +1105,15 @@
         <v>600</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3">
         <v>23</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D25" s="2">
         <v>10</v>
@@ -1086,15 +1125,15 @@
         <v>420</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
         <v>24</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="D26" s="2">
         <v>10</v>
@@ -1106,15 +1145,15 @@
         <v>260</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>25</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="D27" s="2">
         <v>10</v>
@@ -1126,15 +1165,15 @@
         <v>260</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3">
         <v>26</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="D28" s="2">
         <v>5</v>
@@ -1146,15 +1185,15 @@
         <v>260</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3">
         <v>27</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="D29" s="2">
         <v>10</v>
@@ -1166,15 +1205,15 @@
         <v>210</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3">
         <v>28</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="D30" s="2">
         <v>20</v>
@@ -1186,15 +1225,15 @@
         <v>320</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="3">
         <v>29</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D31" s="2">
         <v>5</v>
@@ -1206,15 +1245,15 @@
         <v>350</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3">
         <v>30</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="D32" s="2">
         <v>20</v>
@@ -1226,15 +1265,15 @@
         <v>210</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="3">
         <v>31</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="D33" s="2">
         <v>10</v>
@@ -1246,15 +1285,15 @@
         <v>250</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="3">
         <v>32</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D34" s="2">
         <v>10</v>
@@ -1266,15 +1305,15 @@
         <v>250</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="3">
         <v>33</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D35" s="2">
         <v>5</v>
@@ -1286,15 +1325,15 @@
         <v>500</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="3">
         <v>34</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D36" s="2">
         <v>5</v>
@@ -1306,15 +1345,15 @@
         <v>420</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="3">
         <v>35</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D37" s="2">
         <v>5</v>
@@ -1326,33 +1365,53 @@
         <v>250</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A38" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B38" s="7"/>
-      <c r="C38" s="7"/>
-      <c r="D38" s="7"/>
-      <c r="E38" s="7"/>
-      <c r="F38" s="7"/>
-    </row>
-    <row r="39" spans="1:6" ht="13" x14ac:dyDescent="0.3">
-      <c r="A39" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="B39" s="8"/>
-      <c r="C39" s="8"/>
-      <c r="D39" s="8"/>
-      <c r="E39" s="8"/>
+    <row r="38" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="3">
+        <v>36</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D38" s="2">
+        <v>10</v>
+      </c>
+      <c r="E38" s="2">
+        <v>500</v>
+      </c>
+      <c r="F38" s="2">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B39" s="7"/>
+      <c r="C39" s="7"/>
+      <c r="D39" s="7"/>
+      <c r="E39" s="7"/>
       <c r="F39" s="8"/>
+    </row>
+    <row r="40" spans="1:6" ht="13" x14ac:dyDescent="0.3">
+      <c r="A40" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B40" s="12"/>
+      <c r="C40" s="12"/>
+      <c r="D40" s="12"/>
+      <c r="E40" s="12"/>
+      <c r="F40" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A39:F39"/>
+    <mergeCell ref="A40:F40"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A38:F38"/>
-    <mergeCell ref="A39:F39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="70" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="70" orientation="landscape"/>
 </worksheet>
 </file>
</xml_diff>